<commit_message>
feat(relatorios): aprimora rastreabilidade dos achados individuais
Aplica aos templates dos achados 2 a 6 o padrão de motivos dinâmicos e evidências numeradas adotado no achado 1.

Adiciona regras de motivos do relatório no mapa de verificação para PA02 a PA06, preservando a distinção entre resposta negativa e ajuste decorrente de evidência insuficiente.

Regenera artefatos de execução e comentários do gestor compatíveis com a nova estrutura de rastreabilidade.
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/02-Resultados_Auditoria/tabelas_consolidadas_auditoria.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/02-Resultados_Auditoria/tabelas_consolidadas_auditoria.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6580" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6256" uniqueCount="313">
   <si>
     <t>Nome</t>
   </si>
@@ -6497,13 +6497,7 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>258</v>
-      </c>
       <c r="D2" t="s">
-        <v>258</v>
-      </c>
-      <c r="E2" t="s">
         <v>258</v>
       </c>
       <c r="G2" t="s">
@@ -6612,13 +6606,7 @@
       <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>258</v>
-      </c>
       <c r="D4" t="s">
-        <v>258</v>
-      </c>
-      <c r="E4" t="s">
         <v>258</v>
       </c>
       <c r="G4" t="s">
@@ -6683,16 +6671,10 @@
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>258</v>
-      </c>
       <c r="C5" t="s">
         <v>258</v>
       </c>
       <c r="D5" t="s">
-        <v>258</v>
-      </c>
-      <c r="E5" t="s">
         <v>258</v>
       </c>
       <c r="G5" t="s">
@@ -6760,9 +6742,6 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
-        <v>258</v>
-      </c>
       <c r="C6" t="s">
         <v>258</v>
       </c>
@@ -6770,9 +6749,6 @@
         <v>258</v>
       </c>
       <c r="E6" t="s">
-        <v>258</v>
-      </c>
-      <c r="F6" t="s">
         <v>258</v>
       </c>
       <c r="G6" t="s">
@@ -6905,16 +6881,10 @@
       <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>258</v>
-      </c>
       <c r="E8" t="s">
         <v>258</v>
       </c>
       <c r="F8" t="s">
-        <v>258</v>
-      </c>
-      <c r="G8" t="s">
         <v>258</v>
       </c>
       <c r="H8" t="s">
@@ -6976,9 +6946,6 @@
       <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" t="s">
-        <v>258</v>
-      </c>
       <c r="E9" t="s">
         <v>258</v>
       </c>
@@ -7047,13 +7014,7 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" t="s">
-        <v>258</v>
-      </c>
       <c r="D10" t="s">
-        <v>258</v>
-      </c>
-      <c r="E10" t="s">
         <v>258</v>
       </c>
       <c r="G10" t="s">
@@ -7153,9 +7114,6 @@
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" t="s">
-        <v>258</v>
-      </c>
       <c r="C12" t="s">
         <v>258</v>
       </c>
@@ -7218,9 +7176,6 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
-        <v>258</v>
-      </c>
       <c r="D13" t="s">
         <v>258</v>
       </c>
@@ -7333,13 +7288,7 @@
       <c r="A15" t="s">
         <v>21</v>
       </c>
-      <c r="B15" t="s">
-        <v>258</v>
-      </c>
       <c r="D15" t="s">
-        <v>258</v>
-      </c>
-      <c r="E15" t="s">
         <v>258</v>
       </c>
       <c r="G15" t="s">
@@ -7410,9 +7359,6 @@
       <c r="C16" t="s">
         <v>258</v>
       </c>
-      <c r="F16" t="s">
-        <v>258</v>
-      </c>
       <c r="H16" t="s">
         <v>258</v>
       </c>
@@ -7472,16 +7418,10 @@
       <c r="A17" t="s">
         <v>23</v>
       </c>
-      <c r="B17" t="s">
-        <v>258</v>
-      </c>
       <c r="C17" t="s">
         <v>258</v>
       </c>
       <c r="D17" t="s">
-        <v>258</v>
-      </c>
-      <c r="E17" t="s">
         <v>258</v>
       </c>
       <c r="G17" t="s">
@@ -7608,9 +7548,6 @@
       <c r="A19" t="s">
         <v>25</v>
       </c>
-      <c r="B19" t="s">
-        <v>258</v>
-      </c>
       <c r="C19" t="s">
         <v>258</v>
       </c>
@@ -7618,9 +7555,6 @@
         <v>258</v>
       </c>
       <c r="E19" t="s">
-        <v>258</v>
-      </c>
-      <c r="G19" t="s">
         <v>258</v>
       </c>
       <c r="H19" t="s">
@@ -7664,9 +7598,6 @@
       <c r="A20" t="s">
         <v>26</v>
       </c>
-      <c r="B20" t="s">
-        <v>258</v>
-      </c>
       <c r="C20" t="s">
         <v>258</v>
       </c>
@@ -7729,9 +7660,6 @@
       <c r="A21" t="s">
         <v>28</v>
       </c>
-      <c r="B21" t="s">
-        <v>258</v>
-      </c>
       <c r="C21" t="s">
         <v>258</v>
       </c>
@@ -7806,16 +7734,10 @@
       <c r="A22" t="s">
         <v>29</v>
       </c>
-      <c r="B22" t="s">
-        <v>258</v>
-      </c>
       <c r="C22" t="s">
         <v>258</v>
       </c>
       <c r="D22" t="s">
-        <v>258</v>
-      </c>
-      <c r="E22" t="s">
         <v>258</v>
       </c>
       <c r="G22" t="s">
@@ -7877,16 +7799,7 @@
       <c r="A23" t="s">
         <v>30</v>
       </c>
-      <c r="B23" t="s">
-        <v>258</v>
-      </c>
       <c r="D23" t="s">
-        <v>258</v>
-      </c>
-      <c r="E23" t="s">
-        <v>258</v>
-      </c>
-      <c r="G23" t="s">
         <v>258</v>
       </c>
       <c r="H23" t="s">
@@ -7954,9 +7867,6 @@
       <c r="A24" t="s">
         <v>31</v>
       </c>
-      <c r="B24" t="s">
-        <v>258</v>
-      </c>
       <c r="C24" t="s">
         <v>258</v>
       </c>
@@ -8022,16 +7932,10 @@
       <c r="A25" t="s">
         <v>32</v>
       </c>
-      <c r="B25" t="s">
-        <v>258</v>
-      </c>
       <c r="C25" t="s">
         <v>258</v>
       </c>
       <c r="D25" t="s">
-        <v>258</v>
-      </c>
-      <c r="E25" t="s">
         <v>258</v>
       </c>
       <c r="G25" t="s">
@@ -8099,12 +8003,6 @@
       <c r="A26" t="s">
         <v>33</v>
       </c>
-      <c r="B26" t="s">
-        <v>258</v>
-      </c>
-      <c r="E26" t="s">
-        <v>258</v>
-      </c>
       <c r="G26" t="s">
         <v>258</v>
       </c>
@@ -8179,9 +8077,6 @@
       <c r="F27" t="s">
         <v>258</v>
       </c>
-      <c r="G27" t="s">
-        <v>258</v>
-      </c>
       <c r="H27" t="s">
         <v>258</v>
       </c>
@@ -8226,9 +8121,6 @@
       <c r="A28" t="s">
         <v>35</v>
       </c>
-      <c r="B28" t="s">
-        <v>258</v>
-      </c>
       <c r="C28" t="s">
         <v>258</v>
       </c>
@@ -8297,19 +8189,10 @@
       <c r="A29" t="s">
         <v>36</v>
       </c>
-      <c r="B29" t="s">
-        <v>258</v>
-      </c>
       <c r="C29" t="s">
         <v>258</v>
       </c>
       <c r="D29" t="s">
-        <v>258</v>
-      </c>
-      <c r="E29" t="s">
-        <v>258</v>
-      </c>
-      <c r="G29" t="s">
         <v>258</v>
       </c>
       <c r="H29" t="s">
@@ -8377,9 +8260,6 @@
       <c r="A30" t="s">
         <v>37</v>
       </c>
-      <c r="B30" t="s">
-        <v>258</v>
-      </c>
       <c r="H30" t="s">
         <v>258</v>
       </c>
@@ -8439,13 +8319,7 @@
       <c r="A31" t="s">
         <v>38</v>
       </c>
-      <c r="B31" t="s">
-        <v>258</v>
-      </c>
       <c r="D31" t="s">
-        <v>258</v>
-      </c>
-      <c r="E31" t="s">
         <v>258</v>
       </c>
       <c r="G31" t="s">
@@ -8492,22 +8366,10 @@
       <c r="A32" t="s">
         <v>39</v>
       </c>
-      <c r="B32" t="s">
-        <v>258</v>
-      </c>
       <c r="C32" t="s">
         <v>258</v>
       </c>
       <c r="D32" t="s">
-        <v>258</v>
-      </c>
-      <c r="E32" t="s">
-        <v>258</v>
-      </c>
-      <c r="F32" t="s">
-        <v>258</v>
-      </c>
-      <c r="G32" t="s">
         <v>258</v>
       </c>
       <c r="H32" t="s">
@@ -8575,16 +8437,10 @@
       <c r="A33" t="s">
         <v>40</v>
       </c>
-      <c r="B33" t="s">
-        <v>258</v>
-      </c>
       <c r="C33" t="s">
         <v>258</v>
       </c>
       <c r="D33" t="s">
-        <v>258</v>
-      </c>
-      <c r="E33" t="s">
         <v>258</v>
       </c>
       <c r="G33" t="s">
@@ -8655,9 +8511,6 @@
       <c r="D34" t="s">
         <v>258</v>
       </c>
-      <c r="E34" t="s">
-        <v>258</v>
-      </c>
       <c r="F34" t="s">
         <v>258</v>
       </c>
@@ -8720,9 +8573,6 @@
       <c r="A35" t="s">
         <v>42</v>
       </c>
-      <c r="B35" t="s">
-        <v>258</v>
-      </c>
       <c r="D35" t="s">
         <v>258</v>
       </c>
@@ -8785,9 +8635,6 @@
       <c r="A36" t="s">
         <v>43</v>
       </c>
-      <c r="B36" t="s">
-        <v>258</v>
-      </c>
       <c r="H36" t="s">
         <v>258</v>
       </c>
@@ -8838,9 +8685,6 @@
       <c r="A37" t="s">
         <v>44</v>
       </c>
-      <c r="B37" t="s">
-        <v>258</v>
-      </c>
       <c r="C37" t="s">
         <v>258</v>
       </c>
@@ -8906,13 +8750,7 @@
       <c r="A38" t="s">
         <v>45</v>
       </c>
-      <c r="B38" t="s">
-        <v>258</v>
-      </c>
       <c r="D38" t="s">
-        <v>258</v>
-      </c>
-      <c r="E38" t="s">
         <v>258</v>
       </c>
       <c r="G38" t="s">
@@ -8971,9 +8809,6 @@
       <c r="A39" t="s">
         <v>46</v>
       </c>
-      <c r="B39" t="s">
-        <v>258</v>
-      </c>
       <c r="C39" t="s">
         <v>258</v>
       </c>
@@ -8981,9 +8816,6 @@
         <v>258</v>
       </c>
       <c r="E39" t="s">
-        <v>258</v>
-      </c>
-      <c r="G39" t="s">
         <v>258</v>
       </c>
       <c r="H39" t="s">
@@ -9045,16 +8877,10 @@
       <c r="A40" t="s">
         <v>47</v>
       </c>
-      <c r="B40" t="s">
-        <v>258</v>
-      </c>
       <c r="C40" t="s">
         <v>258</v>
       </c>
       <c r="D40" t="s">
-        <v>258</v>
-      </c>
-      <c r="E40" t="s">
         <v>258</v>
       </c>
       <c r="F40" t="s">
@@ -9157,9 +8983,6 @@
       <c r="A42" t="s">
         <v>49</v>
       </c>
-      <c r="B42" t="s">
-        <v>258</v>
-      </c>
       <c r="C42" t="s">
         <v>258</v>
       </c>
@@ -9260,9 +9083,6 @@
       <c r="A44" t="s">
         <v>52</v>
       </c>
-      <c r="B44" t="s">
-        <v>258</v>
-      </c>
       <c r="H44" t="s">
         <v>258</v>
       </c>
@@ -9292,9 +9112,6 @@
       <c r="A45" t="s">
         <v>53</v>
       </c>
-      <c r="B45" t="s">
-        <v>258</v>
-      </c>
       <c r="C45" t="s">
         <v>258</v>
       </c>
@@ -9366,12 +9183,6 @@
       <c r="A46" t="s">
         <v>54</v>
       </c>
-      <c r="B46" t="s">
-        <v>258</v>
-      </c>
-      <c r="F46" t="s">
-        <v>258</v>
-      </c>
       <c r="H46" t="s">
         <v>258</v>
       </c>
@@ -9404,9 +9215,6 @@
       <c r="A47" t="s">
         <v>55</v>
       </c>
-      <c r="B47" t="s">
-        <v>258</v>
-      </c>
       <c r="D47" t="s">
         <v>258</v>
       </c>
@@ -9463,9 +9271,6 @@
       <c r="A48" t="s">
         <v>56</v>
       </c>
-      <c r="B48" t="s">
-        <v>258</v>
-      </c>
       <c r="C48" t="s">
         <v>258</v>
       </c>
@@ -9543,9 +9348,6 @@
       <c r="D49" t="s">
         <v>258</v>
       </c>
-      <c r="F49" t="s">
-        <v>258</v>
-      </c>
       <c r="H49" t="s">
         <v>258</v>
       </c>
@@ -9593,9 +9395,6 @@
       <c r="A50" t="s">
         <v>58</v>
       </c>
-      <c r="B50" t="s">
-        <v>258</v>
-      </c>
       <c r="C50" t="s">
         <v>258</v>
       </c>
@@ -9603,9 +9402,6 @@
         <v>258</v>
       </c>
       <c r="E50" t="s">
-        <v>258</v>
-      </c>
-      <c r="G50" t="s">
         <v>258</v>
       </c>
       <c r="H50" t="s">
@@ -9670,16 +9466,10 @@
       <c r="A51" t="s">
         <v>59</v>
       </c>
-      <c r="B51" t="s">
-        <v>258</v>
-      </c>
       <c r="C51" t="s">
         <v>258</v>
       </c>
       <c r="D51" t="s">
-        <v>258</v>
-      </c>
-      <c r="E51" t="s">
         <v>258</v>
       </c>
       <c r="G51" t="s">
@@ -9741,13 +9531,7 @@
       <c r="A52" t="s">
         <v>60</v>
       </c>
-      <c r="B52" t="s">
-        <v>258</v>
-      </c>
       <c r="D52" t="s">
-        <v>258</v>
-      </c>
-      <c r="E52" t="s">
         <v>258</v>
       </c>
       <c r="G52" t="s">
@@ -9862,16 +9646,10 @@
       <c r="A54" t="s">
         <v>62</v>
       </c>
-      <c r="B54" t="s">
-        <v>258</v>
-      </c>
       <c r="C54" t="s">
         <v>258</v>
       </c>
       <c r="D54" t="s">
-        <v>258</v>
-      </c>
-      <c r="E54" t="s">
         <v>258</v>
       </c>
       <c r="G54" t="s">
@@ -9939,12 +9717,6 @@
       <c r="A55" t="s">
         <v>63</v>
       </c>
-      <c r="B55" t="s">
-        <v>258</v>
-      </c>
-      <c r="E55" t="s">
-        <v>258</v>
-      </c>
       <c r="G55" t="s">
         <v>258</v>
       </c>
@@ -9995,12 +9767,6 @@
       <c r="A56" t="s">
         <v>65</v>
       </c>
-      <c r="B56" t="s">
-        <v>258</v>
-      </c>
-      <c r="F56" t="s">
-        <v>258</v>
-      </c>
       <c r="H56" t="s">
         <v>258</v>
       </c>
@@ -10048,9 +9814,6 @@
       <c r="A57" t="s">
         <v>66</v>
       </c>
-      <c r="B57" t="s">
-        <v>258</v>
-      </c>
       <c r="D57" t="s">
         <v>258</v>
       </c>
@@ -10113,9 +9876,6 @@
       <c r="A58" t="s">
         <v>67</v>
       </c>
-      <c r="B58" t="s">
-        <v>258</v>
-      </c>
       <c r="C58" t="s">
         <v>258</v>
       </c>
@@ -10243,16 +10003,10 @@
       <c r="A60" t="s">
         <v>69</v>
       </c>
-      <c r="B60" t="s">
-        <v>258</v>
-      </c>
       <c r="C60" t="s">
         <v>258</v>
       </c>
       <c r="D60" t="s">
-        <v>258</v>
-      </c>
-      <c r="E60" t="s">
         <v>258</v>
       </c>
       <c r="G60" t="s">
@@ -10314,9 +10068,6 @@
       <c r="A61" t="s">
         <v>70</v>
       </c>
-      <c r="B61" t="s">
-        <v>258</v>
-      </c>
       <c r="C61" t="s">
         <v>258</v>
       </c>
@@ -10382,9 +10133,6 @@
       <c r="D62" t="s">
         <v>258</v>
       </c>
-      <c r="E62" t="s">
-        <v>258</v>
-      </c>
       <c r="F62" t="s">
         <v>258</v>
       </c>
@@ -10450,9 +10198,6 @@
       <c r="D63" t="s">
         <v>258</v>
       </c>
-      <c r="E63" t="s">
-        <v>258</v>
-      </c>
       <c r="G63" t="s">
         <v>258</v>
       </c>
@@ -10506,13 +10251,7 @@
       <c r="A64" t="s">
         <v>73</v>
       </c>
-      <c r="B64" t="s">
-        <v>258</v>
-      </c>
       <c r="D64" t="s">
-        <v>258</v>
-      </c>
-      <c r="E64" t="s">
         <v>258</v>
       </c>
       <c r="G64" t="s">
@@ -10577,9 +10316,6 @@
       <c r="A65" t="s">
         <v>74</v>
       </c>
-      <c r="B65" t="s">
-        <v>258</v>
-      </c>
       <c r="D65" t="s">
         <v>258</v>
       </c>
@@ -10645,16 +10381,10 @@
       <c r="A66" t="s">
         <v>75</v>
       </c>
-      <c r="B66" t="s">
-        <v>258</v>
-      </c>
       <c r="C66" t="s">
         <v>258</v>
       </c>
       <c r="D66" t="s">
-        <v>258</v>
-      </c>
-      <c r="E66" t="s">
         <v>258</v>
       </c>
       <c r="G66" t="s">
@@ -10716,9 +10446,6 @@
       <c r="A67" t="s">
         <v>76</v>
       </c>
-      <c r="E67" t="s">
-        <v>258</v>
-      </c>
       <c r="G67" t="s">
         <v>258</v>
       </c>
@@ -10748,13 +10475,7 @@
       <c r="A68" t="s">
         <v>77</v>
       </c>
-      <c r="B68" t="s">
-        <v>258</v>
-      </c>
       <c r="D68" t="s">
-        <v>258</v>
-      </c>
-      <c r="E68" t="s">
         <v>258</v>
       </c>
       <c r="G68" t="s">
@@ -10828,9 +10549,6 @@
       <c r="E69" t="s">
         <v>258</v>
       </c>
-      <c r="F69" t="s">
-        <v>258</v>
-      </c>
       <c r="G69" t="s">
         <v>258</v>
       </c>
@@ -10949,12 +10667,6 @@
       <c r="E71" t="s">
         <v>258</v>
       </c>
-      <c r="F71" t="s">
-        <v>258</v>
-      </c>
-      <c r="G71" t="s">
-        <v>258</v>
-      </c>
       <c r="H71" t="s">
         <v>258</v>
       </c>
@@ -10990,9 +10702,6 @@
       <c r="D72" t="s">
         <v>258</v>
       </c>
-      <c r="E72" t="s">
-        <v>258</v>
-      </c>
       <c r="G72" t="s">
         <v>258</v>
       </c>
@@ -11061,9 +10770,6 @@
       <c r="D73" t="s">
         <v>258</v>
       </c>
-      <c r="E73" t="s">
-        <v>258</v>
-      </c>
       <c r="G73" t="s">
         <v>258</v>
       </c>
@@ -11123,9 +10829,6 @@
       <c r="A74" t="s">
         <v>85</v>
       </c>
-      <c r="B74" t="s">
-        <v>258</v>
-      </c>
       <c r="C74" t="s">
         <v>258</v>
       </c>
@@ -11194,16 +10897,10 @@
       <c r="A75" t="s">
         <v>86</v>
       </c>
-      <c r="B75" t="s">
-        <v>258</v>
-      </c>
       <c r="C75" t="s">
         <v>258</v>
       </c>
       <c r="D75" t="s">
-        <v>258</v>
-      </c>
-      <c r="E75" t="s">
         <v>258</v>
       </c>
       <c r="G75" t="s">
@@ -11268,9 +10965,6 @@
       <c r="B76" t="s">
         <v>258</v>
       </c>
-      <c r="E76" t="s">
-        <v>258</v>
-      </c>
       <c r="G76" t="s">
         <v>258</v>
       </c>
@@ -11359,22 +11053,10 @@
       <c r="A78" t="s">
         <v>89</v>
       </c>
-      <c r="B78" t="s">
-        <v>258</v>
-      </c>
       <c r="C78" t="s">
         <v>258</v>
       </c>
       <c r="D78" t="s">
-        <v>258</v>
-      </c>
-      <c r="E78" t="s">
-        <v>258</v>
-      </c>
-      <c r="F78" t="s">
-        <v>258</v>
-      </c>
-      <c r="G78" t="s">
         <v>258</v>
       </c>
       <c r="H78" t="s">
@@ -11442,9 +11124,6 @@
       <c r="A79" t="s">
         <v>90</v>
       </c>
-      <c r="B79" t="s">
-        <v>258</v>
-      </c>
       <c r="D79" t="s">
         <v>258</v>
       </c>
@@ -11510,9 +11189,6 @@
       <c r="A80" t="s">
         <v>91</v>
       </c>
-      <c r="B80" t="s">
-        <v>258</v>
-      </c>
       <c r="D80" t="s">
         <v>258</v>
       </c>
@@ -11575,12 +11251,6 @@
       <c r="A81" t="s">
         <v>92</v>
       </c>
-      <c r="B81" t="s">
-        <v>258</v>
-      </c>
-      <c r="E81" t="s">
-        <v>258</v>
-      </c>
       <c r="G81" t="s">
         <v>258</v>
       </c>
@@ -11646,16 +11316,7 @@
       <c r="A82" t="s">
         <v>93</v>
       </c>
-      <c r="B82" t="s">
-        <v>258</v>
-      </c>
       <c r="D82" t="s">
-        <v>258</v>
-      </c>
-      <c r="E82" t="s">
-        <v>258</v>
-      </c>
-      <c r="G82" t="s">
         <v>258</v>
       </c>
       <c r="H82" t="s">
@@ -11723,9 +11384,6 @@
       <c r="A83" t="s">
         <v>94</v>
       </c>
-      <c r="B83" t="s">
-        <v>258</v>
-      </c>
       <c r="C83" t="s">
         <v>258</v>
       </c>
@@ -11733,9 +11391,6 @@
         <v>258</v>
       </c>
       <c r="E83" t="s">
-        <v>258</v>
-      </c>
-      <c r="F83" t="s">
         <v>258</v>
       </c>
       <c r="G83" t="s">
@@ -11812,9 +11467,6 @@
       <c r="D84" t="s">
         <v>258</v>
       </c>
-      <c r="E84" t="s">
-        <v>258</v>
-      </c>
       <c r="G84" t="s">
         <v>258</v>
       </c>
@@ -11874,9 +11526,6 @@
       <c r="A85" t="s">
         <v>96</v>
       </c>
-      <c r="B85" t="s">
-        <v>258</v>
-      </c>
       <c r="C85" t="s">
         <v>258</v>
       </c>
@@ -11945,9 +11594,6 @@
       <c r="A86" t="s">
         <v>97</v>
       </c>
-      <c r="B86" t="s">
-        <v>258</v>
-      </c>
       <c r="D86" t="s">
         <v>258</v>
       </c>
@@ -12010,13 +11656,7 @@
       <c r="A87" t="s">
         <v>98</v>
       </c>
-      <c r="B87" t="s">
-        <v>258</v>
-      </c>
       <c r="D87" t="s">
-        <v>258</v>
-      </c>
-      <c r="E87" t="s">
         <v>258</v>
       </c>
       <c r="G87" t="s">
@@ -12084,9 +11724,6 @@
       <c r="A88" t="s">
         <v>99</v>
       </c>
-      <c r="B88" t="s">
-        <v>258</v>
-      </c>
       <c r="H88" t="s">
         <v>258</v>
       </c>
@@ -12143,9 +11780,6 @@
       <c r="A89" t="s">
         <v>100</v>
       </c>
-      <c r="B89" t="s">
-        <v>258</v>
-      </c>
       <c r="C89" t="s">
         <v>258</v>
       </c>
@@ -12208,16 +11842,10 @@
       <c r="A90" t="s">
         <v>101</v>
       </c>
-      <c r="B90" t="s">
-        <v>258</v>
-      </c>
       <c r="C90" t="s">
         <v>258</v>
       </c>
       <c r="D90" t="s">
-        <v>258</v>
-      </c>
-      <c r="E90" t="s">
         <v>258</v>
       </c>
       <c r="G90" t="s">
@@ -12353,9 +11981,6 @@
       <c r="A92" t="s">
         <v>103</v>
       </c>
-      <c r="B92" t="s">
-        <v>258</v>
-      </c>
       <c r="C92" t="s">
         <v>258</v>
       </c>
@@ -12415,9 +12040,6 @@
       <c r="A93" t="s">
         <v>104</v>
       </c>
-      <c r="B93" t="s">
-        <v>258</v>
-      </c>
       <c r="C93" t="s">
         <v>258</v>
       </c>
@@ -12554,13 +12176,7 @@
       <c r="A95" t="s">
         <v>106</v>
       </c>
-      <c r="B95" t="s">
-        <v>258</v>
-      </c>
       <c r="D95" t="s">
-        <v>258</v>
-      </c>
-      <c r="E95" t="s">
         <v>258</v>
       </c>
       <c r="G95" t="s">
@@ -12628,9 +12244,6 @@
       <c r="A96" t="s">
         <v>107</v>
       </c>
-      <c r="B96" t="s">
-        <v>258</v>
-      </c>
       <c r="D96" t="s">
         <v>258</v>
       </c>
@@ -12690,16 +12303,10 @@
       <c r="A97" t="s">
         <v>108</v>
       </c>
-      <c r="B97" t="s">
-        <v>258</v>
-      </c>
       <c r="E97" t="s">
         <v>258</v>
       </c>
       <c r="F97" t="s">
-        <v>258</v>
-      </c>
-      <c r="G97" t="s">
         <v>258</v>
       </c>
       <c r="H97" t="s">
@@ -12758,9 +12365,6 @@
       <c r="A98" t="s">
         <v>109</v>
       </c>
-      <c r="B98" t="s">
-        <v>258</v>
-      </c>
       <c r="D98" t="s">
         <v>258</v>
       </c>
@@ -12811,16 +12415,10 @@
       <c r="A99" t="s">
         <v>110</v>
       </c>
-      <c r="B99" t="s">
-        <v>258</v>
-      </c>
       <c r="C99" t="s">
         <v>258</v>
       </c>
       <c r="D99" t="s">
-        <v>258</v>
-      </c>
-      <c r="E99" t="s">
         <v>258</v>
       </c>
       <c r="G99" t="s">
@@ -12897,9 +12495,6 @@
       <c r="D100" t="s">
         <v>258</v>
       </c>
-      <c r="E100" t="s">
-        <v>258</v>
-      </c>
       <c r="G100" t="s">
         <v>258</v>
       </c>
@@ -12956,16 +12551,10 @@
       <c r="A101" t="s">
         <v>112</v>
       </c>
-      <c r="B101" t="s">
-        <v>258</v>
-      </c>
       <c r="C101" t="s">
         <v>258</v>
       </c>
       <c r="D101" t="s">
-        <v>258</v>
-      </c>
-      <c r="F101" t="s">
         <v>258</v>
       </c>
       <c r="H101" t="s">
@@ -13030,9 +12619,6 @@
       <c r="A102" t="s">
         <v>113</v>
       </c>
-      <c r="B102" t="s">
-        <v>258</v>
-      </c>
       <c r="C102" t="s">
         <v>258</v>
       </c>
@@ -13104,16 +12690,10 @@
       <c r="A103" t="s">
         <v>114</v>
       </c>
-      <c r="B103" t="s">
-        <v>258</v>
-      </c>
       <c r="C103" t="s">
         <v>258</v>
       </c>
       <c r="D103" t="s">
-        <v>258</v>
-      </c>
-      <c r="E103" t="s">
         <v>258</v>
       </c>
       <c r="G103" t="s">
@@ -13181,16 +12761,10 @@
       <c r="A104" t="s">
         <v>115</v>
       </c>
-      <c r="B104" t="s">
-        <v>258</v>
-      </c>
       <c r="C104" t="s">
         <v>258</v>
       </c>
       <c r="D104" t="s">
-        <v>258</v>
-      </c>
-      <c r="E104" t="s">
         <v>258</v>
       </c>
       <c r="G104" t="s">
@@ -13252,13 +12826,7 @@
       <c r="A105" t="s">
         <v>116</v>
       </c>
-      <c r="B105" t="s">
-        <v>258</v>
-      </c>
       <c r="E105" t="s">
-        <v>258</v>
-      </c>
-      <c r="G105" t="s">
         <v>258</v>
       </c>
       <c r="H105" t="s">
@@ -13311,9 +12879,6 @@
       <c r="A106" t="s">
         <v>117</v>
       </c>
-      <c r="B106" t="s">
-        <v>258</v>
-      </c>
       <c r="C106" t="s">
         <v>258</v>
       </c>
@@ -13435,16 +13000,10 @@
       <c r="A108" t="s">
         <v>119</v>
       </c>
-      <c r="B108" t="s">
-        <v>258</v>
-      </c>
       <c r="C108" t="s">
         <v>258</v>
       </c>
       <c r="D108" t="s">
-        <v>258</v>
-      </c>
-      <c r="E108" t="s">
         <v>258</v>
       </c>
       <c r="G108" t="s">
@@ -13509,19 +13068,10 @@
       <c r="A109" t="s">
         <v>120</v>
       </c>
-      <c r="B109" t="s">
-        <v>258</v>
-      </c>
       <c r="C109" t="s">
         <v>258</v>
       </c>
       <c r="D109" t="s">
-        <v>258</v>
-      </c>
-      <c r="E109" t="s">
-        <v>258</v>
-      </c>
-      <c r="G109" t="s">
         <v>258</v>
       </c>
       <c r="H109" t="s">
@@ -13589,16 +13139,10 @@
       <c r="A110" t="s">
         <v>121</v>
       </c>
-      <c r="B110" t="s">
-        <v>258</v>
-      </c>
       <c r="C110" t="s">
         <v>258</v>
       </c>
       <c r="D110" t="s">
-        <v>258</v>
-      </c>
-      <c r="E110" t="s">
         <v>258</v>
       </c>
       <c r="G110" t="s">
@@ -13734,16 +13278,10 @@
       <c r="A112" t="s">
         <v>123</v>
       </c>
-      <c r="B112" t="s">
-        <v>258</v>
-      </c>
       <c r="C112" t="s">
         <v>258</v>
       </c>
       <c r="D112" t="s">
-        <v>258</v>
-      </c>
-      <c r="E112" t="s">
         <v>258</v>
       </c>
       <c r="F112" t="s">
@@ -13814,16 +13352,10 @@
       <c r="A113" t="s">
         <v>124</v>
       </c>
-      <c r="B113" t="s">
-        <v>258</v>
-      </c>
       <c r="C113" t="s">
         <v>258</v>
       </c>
       <c r="D113" t="s">
-        <v>258</v>
-      </c>
-      <c r="E113" t="s">
         <v>258</v>
       </c>
       <c r="G113" t="s">
@@ -13891,16 +13423,7 @@
       <c r="A114" t="s">
         <v>125</v>
       </c>
-      <c r="B114" t="s">
-        <v>258</v>
-      </c>
       <c r="D114" t="s">
-        <v>258</v>
-      </c>
-      <c r="E114" t="s">
-        <v>258</v>
-      </c>
-      <c r="F114" t="s">
         <v>258</v>
       </c>
       <c r="G114" t="s">
@@ -13962,19 +13485,10 @@
       <c r="A115" t="s">
         <v>126</v>
       </c>
-      <c r="B115" t="s">
-        <v>258</v>
-      </c>
       <c r="C115" t="s">
         <v>258</v>
       </c>
       <c r="D115" t="s">
-        <v>258</v>
-      </c>
-      <c r="E115" t="s">
-        <v>258</v>
-      </c>
-      <c r="F115" t="s">
         <v>258</v>
       </c>
       <c r="G115" t="s">
@@ -14135,13 +13649,7 @@
       <c r="C2" t="s">
         <v>258</v>
       </c>
-      <c r="D2" t="s">
-        <v>258</v>
-      </c>
       <c r="E2" t="s">
-        <v>258</v>
-      </c>
-      <c r="G2" t="s">
         <v>258</v>
       </c>
       <c r="K2" t="s">
@@ -14250,16 +13758,10 @@
       <c r="C4" t="s">
         <v>258</v>
       </c>
-      <c r="D4" t="s">
-        <v>258</v>
-      </c>
       <c r="E4" t="s">
         <v>258</v>
       </c>
       <c r="F4" t="s">
-        <v>258</v>
-      </c>
-      <c r="G4" t="s">
         <v>258</v>
       </c>
       <c r="H4" t="s">
@@ -14321,16 +13823,10 @@
       <c r="C5" t="s">
         <v>258</v>
       </c>
-      <c r="D5" t="s">
-        <v>258</v>
-      </c>
       <c r="E5" t="s">
         <v>258</v>
       </c>
       <c r="F5" t="s">
-        <v>258</v>
-      </c>
-      <c r="G5" t="s">
         <v>258</v>
       </c>
       <c r="H5" t="s">
@@ -14407,9 +13903,6 @@
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" t="s">
-        <v>258</v>
-      </c>
       <c r="H6" t="s">
         <v>258</v>
       </c>
@@ -14438,9 +13931,6 @@
         <v>258</v>
       </c>
       <c r="Q6" t="s">
-        <v>258</v>
-      </c>
-      <c r="R6" t="s">
         <v>258</v>
       </c>
       <c r="S6" t="s">
@@ -14540,9 +14030,6 @@
       <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
-        <v>258</v>
-      </c>
       <c r="D8" t="s">
         <v>258</v>
       </c>
@@ -14550,9 +14037,6 @@
         <v>258</v>
       </c>
       <c r="F8" t="s">
-        <v>258</v>
-      </c>
-      <c r="G8" t="s">
         <v>258</v>
       </c>
       <c r="H8" t="s">
@@ -14623,9 +14107,6 @@
       <c r="F9" t="s">
         <v>258</v>
       </c>
-      <c r="G9" t="s">
-        <v>258</v>
-      </c>
       <c r="H9" t="s">
         <v>258</v>
       </c>
@@ -14685,16 +14166,10 @@
       <c r="C10" t="s">
         <v>258</v>
       </c>
-      <c r="D10" t="s">
-        <v>258</v>
-      </c>
       <c r="E10" t="s">
         <v>258</v>
       </c>
       <c r="F10" t="s">
-        <v>258</v>
-      </c>
-      <c r="G10" t="s">
         <v>258</v>
       </c>
       <c r="K10" t="s">
@@ -14791,9 +14266,6 @@
       <c r="E12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" t="s">
-        <v>258</v>
-      </c>
       <c r="H12" t="s">
         <v>258</v>
       </c>
@@ -14865,9 +14337,6 @@
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" t="s">
-        <v>258</v>
-      </c>
       <c r="K13" t="s">
         <v>258</v>
       </c>
@@ -14971,16 +14440,10 @@
       <c r="C15" t="s">
         <v>258</v>
       </c>
-      <c r="D15" t="s">
-        <v>258</v>
-      </c>
       <c r="E15" t="s">
         <v>258</v>
       </c>
       <c r="F15" t="s">
-        <v>258</v>
-      </c>
-      <c r="G15" t="s">
         <v>258</v>
       </c>
       <c r="H15" t="s">
@@ -15075,9 +14538,6 @@
       <c r="Q16" t="s">
         <v>258</v>
       </c>
-      <c r="R16" t="s">
-        <v>258</v>
-      </c>
       <c r="S16" t="s">
         <v>258</v>
       </c>
@@ -15110,16 +14570,10 @@
       <c r="C17" t="s">
         <v>258</v>
       </c>
-      <c r="D17" t="s">
-        <v>258</v>
-      </c>
       <c r="E17" t="s">
         <v>258</v>
       </c>
       <c r="F17" t="s">
-        <v>258</v>
-      </c>
-      <c r="G17" t="s">
         <v>258</v>
       </c>
       <c r="H17" t="s">
@@ -15243,9 +14697,6 @@
       <c r="A19" t="s">
         <v>25</v>
       </c>
-      <c r="C19" t="s">
-        <v>258</v>
-      </c>
       <c r="D19" t="s">
         <v>258</v>
       </c>
@@ -15253,9 +14704,6 @@
         <v>258</v>
       </c>
       <c r="F19" t="s">
-        <v>258</v>
-      </c>
-      <c r="G19" t="s">
         <v>258</v>
       </c>
       <c r="H19" t="s">
@@ -15305,9 +14753,6 @@
       <c r="F20" t="s">
         <v>258</v>
       </c>
-      <c r="G20" t="s">
-        <v>258</v>
-      </c>
       <c r="H20" t="s">
         <v>258</v>
       </c>
@@ -15376,9 +14821,6 @@
       <c r="F21" t="s">
         <v>258</v>
       </c>
-      <c r="G21" t="s">
-        <v>258</v>
-      </c>
       <c r="H21" t="s">
         <v>258</v>
       </c>
@@ -15444,16 +14886,10 @@
       <c r="C22" t="s">
         <v>258</v>
       </c>
-      <c r="D22" t="s">
-        <v>258</v>
-      </c>
       <c r="E22" t="s">
         <v>258</v>
       </c>
       <c r="F22" t="s">
-        <v>258</v>
-      </c>
-      <c r="G22" t="s">
         <v>258</v>
       </c>
       <c r="H22" t="s">
@@ -15515,19 +14951,10 @@
       <c r="B23" t="s">
         <v>258</v>
       </c>
-      <c r="C23" t="s">
-        <v>258</v>
-      </c>
-      <c r="D23" t="s">
-        <v>258</v>
-      </c>
       <c r="E23" t="s">
         <v>258</v>
       </c>
       <c r="F23" t="s">
-        <v>258</v>
-      </c>
-      <c r="G23" t="s">
         <v>258</v>
       </c>
       <c r="H23" t="s">
@@ -15601,9 +15028,6 @@
       <c r="F24" t="s">
         <v>258</v>
       </c>
-      <c r="G24" t="s">
-        <v>258</v>
-      </c>
       <c r="H24" t="s">
         <v>258</v>
       </c>
@@ -15660,16 +15084,10 @@
       <c r="C25" t="s">
         <v>258</v>
       </c>
-      <c r="D25" t="s">
-        <v>258</v>
-      </c>
       <c r="E25" t="s">
         <v>258</v>
       </c>
       <c r="F25" t="s">
-        <v>258</v>
-      </c>
-      <c r="G25" t="s">
         <v>258</v>
       </c>
       <c r="H25" t="s">
@@ -15737,16 +15155,10 @@
       <c r="C26" t="s">
         <v>258</v>
       </c>
-      <c r="D26" t="s">
-        <v>258</v>
-      </c>
       <c r="E26" t="s">
         <v>258</v>
       </c>
       <c r="F26" t="s">
-        <v>258</v>
-      </c>
-      <c r="G26" t="s">
         <v>258</v>
       </c>
       <c r="H26" t="s">
@@ -15799,9 +15211,6 @@
       <c r="A27" t="s">
         <v>34</v>
       </c>
-      <c r="C27" t="s">
-        <v>258</v>
-      </c>
       <c r="D27" t="s">
         <v>258</v>
       </c>
@@ -15873,9 +15282,6 @@
       <c r="F28" t="s">
         <v>258</v>
       </c>
-      <c r="G28" t="s">
-        <v>258</v>
-      </c>
       <c r="H28" t="s">
         <v>258</v>
       </c>
@@ -15935,19 +15341,10 @@
       <c r="B29" t="s">
         <v>258</v>
       </c>
-      <c r="C29" t="s">
-        <v>258</v>
-      </c>
-      <c r="D29" t="s">
-        <v>258</v>
-      </c>
       <c r="E29" t="s">
         <v>258</v>
       </c>
       <c r="F29" t="s">
-        <v>258</v>
-      </c>
-      <c r="G29" t="s">
         <v>258</v>
       </c>
       <c r="H29" t="s">
@@ -16018,9 +15415,6 @@
       <c r="F30" t="s">
         <v>258</v>
       </c>
-      <c r="G30" t="s">
-        <v>258</v>
-      </c>
       <c r="H30" t="s">
         <v>258</v>
       </c>
@@ -16077,16 +15471,10 @@
       <c r="C31" t="s">
         <v>258</v>
       </c>
-      <c r="D31" t="s">
-        <v>258</v>
-      </c>
       <c r="E31" t="s">
         <v>258</v>
       </c>
       <c r="F31" t="s">
-        <v>258</v>
-      </c>
-      <c r="G31" t="s">
         <v>258</v>
       </c>
       <c r="K31" t="s">
@@ -16130,21 +15518,12 @@
       <c r="B32" t="s">
         <v>258</v>
       </c>
-      <c r="C32" t="s">
-        <v>258</v>
-      </c>
-      <c r="D32" t="s">
-        <v>258</v>
-      </c>
       <c r="E32" t="s">
         <v>258</v>
       </c>
       <c r="F32" t="s">
         <v>258</v>
       </c>
-      <c r="G32" t="s">
-        <v>258</v>
-      </c>
       <c r="H32" t="s">
         <v>258</v>
       </c>
@@ -16173,9 +15552,6 @@
         <v>258</v>
       </c>
       <c r="Q32" t="s">
-        <v>258</v>
-      </c>
-      <c r="R32" t="s">
         <v>258</v>
       </c>
       <c r="S32" t="s">
@@ -16213,16 +15589,10 @@
       <c r="C33" t="s">
         <v>258</v>
       </c>
-      <c r="D33" t="s">
-        <v>258</v>
-      </c>
       <c r="E33" t="s">
         <v>258</v>
       </c>
       <c r="F33" t="s">
-        <v>258</v>
-      </c>
-      <c r="G33" t="s">
         <v>258</v>
       </c>
       <c r="H33" t="s">
@@ -16284,9 +15654,6 @@
       <c r="C34" t="s">
         <v>258</v>
       </c>
-      <c r="D34" t="s">
-        <v>258</v>
-      </c>
       <c r="E34" t="s">
         <v>258</v>
       </c>
@@ -16361,9 +15728,6 @@
       <c r="F35" t="s">
         <v>258</v>
       </c>
-      <c r="G35" t="s">
-        <v>258</v>
-      </c>
       <c r="H35" t="s">
         <v>258</v>
       </c>
@@ -16426,9 +15790,6 @@
       <c r="F36" t="s">
         <v>258</v>
       </c>
-      <c r="G36" t="s">
-        <v>258</v>
-      </c>
       <c r="H36" t="s">
         <v>258</v>
       </c>
@@ -16479,9 +15840,6 @@
       <c r="F37" t="s">
         <v>258</v>
       </c>
-      <c r="G37" t="s">
-        <v>258</v>
-      </c>
       <c r="H37" t="s">
         <v>258</v>
       </c>
@@ -16544,16 +15902,10 @@
       <c r="C38" t="s">
         <v>258</v>
       </c>
-      <c r="D38" t="s">
-        <v>258</v>
-      </c>
       <c r="E38" t="s">
         <v>258</v>
       </c>
       <c r="F38" t="s">
-        <v>258</v>
-      </c>
-      <c r="G38" t="s">
         <v>258</v>
       </c>
       <c r="H38" t="s">
@@ -16606,9 +15958,6 @@
       <c r="A39" t="s">
         <v>46</v>
       </c>
-      <c r="C39" t="s">
-        <v>258</v>
-      </c>
       <c r="D39" t="s">
         <v>258</v>
       </c>
@@ -16616,9 +15965,6 @@
         <v>258</v>
       </c>
       <c r="F39" t="s">
-        <v>258</v>
-      </c>
-      <c r="G39" t="s">
         <v>258</v>
       </c>
       <c r="H39" t="s">
@@ -16683,16 +16029,10 @@
       <c r="C40" t="s">
         <v>258</v>
       </c>
-      <c r="D40" t="s">
-        <v>258</v>
-      </c>
       <c r="E40" t="s">
         <v>258</v>
       </c>
       <c r="F40" t="s">
-        <v>258</v>
-      </c>
-      <c r="G40" t="s">
         <v>258</v>
       </c>
       <c r="H40" t="s">
@@ -16798,9 +16138,6 @@
       <c r="F42" t="s">
         <v>258</v>
       </c>
-      <c r="G42" t="s">
-        <v>258</v>
-      </c>
       <c r="H42" t="s">
         <v>258</v>
       </c>
@@ -16898,9 +16235,6 @@
       <c r="E44" t="s">
         <v>258</v>
       </c>
-      <c r="G44" t="s">
-        <v>258</v>
-      </c>
       <c r="N44" t="s">
         <v>258</v>
       </c>
@@ -16939,9 +16273,6 @@
       <c r="F45" t="s">
         <v>258</v>
       </c>
-      <c r="G45" t="s">
-        <v>258</v>
-      </c>
       <c r="H45" t="s">
         <v>258</v>
       </c>
@@ -17004,9 +16335,6 @@
       <c r="E46" t="s">
         <v>258</v>
       </c>
-      <c r="G46" t="s">
-        <v>258</v>
-      </c>
       <c r="N46" t="s">
         <v>258</v>
       </c>
@@ -17014,9 +16342,6 @@
         <v>258</v>
       </c>
       <c r="Q46" t="s">
-        <v>258</v>
-      </c>
-      <c r="R46" t="s">
         <v>258</v>
       </c>
       <c r="S46" t="s">
@@ -17045,9 +16370,6 @@
       <c r="F47" t="s">
         <v>258</v>
       </c>
-      <c r="G47" t="s">
-        <v>258</v>
-      </c>
       <c r="I47" t="s">
         <v>258</v>
       </c>
@@ -17110,9 +16432,6 @@
       <c r="F48" t="s">
         <v>258</v>
       </c>
-      <c r="G48" t="s">
-        <v>258</v>
-      </c>
       <c r="H48" t="s">
         <v>258</v>
       </c>
@@ -17196,9 +16515,6 @@
       <c r="Q49" t="s">
         <v>258</v>
       </c>
-      <c r="R49" t="s">
-        <v>258</v>
-      </c>
       <c r="S49" t="s">
         <v>258</v>
       </c>
@@ -17228,9 +16544,6 @@
       <c r="A50" t="s">
         <v>58</v>
       </c>
-      <c r="C50" t="s">
-        <v>258</v>
-      </c>
       <c r="D50" t="s">
         <v>258</v>
       </c>
@@ -17238,9 +16551,6 @@
         <v>258</v>
       </c>
       <c r="F50" t="s">
-        <v>258</v>
-      </c>
-      <c r="G50" t="s">
         <v>258</v>
       </c>
       <c r="H50" t="s">
@@ -17308,16 +16618,10 @@
       <c r="C51" t="s">
         <v>258</v>
       </c>
-      <c r="D51" t="s">
-        <v>258</v>
-      </c>
       <c r="E51" t="s">
         <v>258</v>
       </c>
       <c r="F51" t="s">
-        <v>258</v>
-      </c>
-      <c r="G51" t="s">
         <v>258</v>
       </c>
       <c r="H51" t="s">
@@ -17379,16 +16683,10 @@
       <c r="C52" t="s">
         <v>258</v>
       </c>
-      <c r="D52" t="s">
-        <v>258</v>
-      </c>
       <c r="E52" t="s">
         <v>258</v>
       </c>
       <c r="F52" t="s">
-        <v>258</v>
-      </c>
-      <c r="G52" t="s">
         <v>258</v>
       </c>
       <c r="H52" t="s">
@@ -17500,16 +16798,10 @@
       <c r="C54" t="s">
         <v>258</v>
       </c>
-      <c r="D54" t="s">
-        <v>258</v>
-      </c>
       <c r="E54" t="s">
         <v>258</v>
       </c>
       <c r="F54" t="s">
-        <v>258</v>
-      </c>
-      <c r="G54" t="s">
         <v>258</v>
       </c>
       <c r="H54" t="s">
@@ -17577,16 +16869,10 @@
       <c r="C55" t="s">
         <v>258</v>
       </c>
-      <c r="D55" t="s">
-        <v>258</v>
-      </c>
       <c r="E55" t="s">
         <v>258</v>
       </c>
       <c r="F55" t="s">
-        <v>258</v>
-      </c>
-      <c r="G55" t="s">
         <v>258</v>
       </c>
       <c r="H55" t="s">
@@ -17636,9 +16922,6 @@
       <c r="F56" t="s">
         <v>258</v>
       </c>
-      <c r="G56" t="s">
-        <v>258</v>
-      </c>
       <c r="H56" t="s">
         <v>258</v>
       </c>
@@ -17652,9 +16935,6 @@
         <v>258</v>
       </c>
       <c r="Q56" t="s">
-        <v>258</v>
-      </c>
-      <c r="R56" t="s">
         <v>258</v>
       </c>
       <c r="S56" t="s">
@@ -17689,9 +16969,6 @@
       <c r="F57" t="s">
         <v>258</v>
       </c>
-      <c r="G57" t="s">
-        <v>258</v>
-      </c>
       <c r="H57" t="s">
         <v>258</v>
       </c>
@@ -17760,9 +17037,6 @@
       <c r="F58" t="s">
         <v>258</v>
       </c>
-      <c r="G58" t="s">
-        <v>258</v>
-      </c>
       <c r="H58" t="s">
         <v>258</v>
       </c>
@@ -17881,16 +17155,10 @@
       <c r="C60" t="s">
         <v>258</v>
       </c>
-      <c r="D60" t="s">
-        <v>258</v>
-      </c>
       <c r="E60" t="s">
         <v>258</v>
       </c>
       <c r="F60" t="s">
-        <v>258</v>
-      </c>
-      <c r="G60" t="s">
         <v>258</v>
       </c>
       <c r="H60" t="s">
@@ -17955,9 +17223,6 @@
       <c r="F61" t="s">
         <v>258</v>
       </c>
-      <c r="G61" t="s">
-        <v>258</v>
-      </c>
       <c r="H61" t="s">
         <v>258</v>
       </c>
@@ -18014,9 +17279,6 @@
       <c r="C62" t="s">
         <v>258</v>
       </c>
-      <c r="D62" t="s">
-        <v>258</v>
-      </c>
       <c r="E62" t="s">
         <v>258</v>
       </c>
@@ -18082,9 +17344,6 @@
       <c r="C63" t="s">
         <v>258</v>
       </c>
-      <c r="D63" t="s">
-        <v>258</v>
-      </c>
       <c r="E63" t="s">
         <v>258</v>
       </c>
@@ -18144,16 +17403,10 @@
       <c r="C64" t="s">
         <v>258</v>
       </c>
-      <c r="D64" t="s">
-        <v>258</v>
-      </c>
       <c r="E64" t="s">
         <v>258</v>
       </c>
       <c r="F64" t="s">
-        <v>258</v>
-      </c>
-      <c r="G64" t="s">
         <v>258</v>
       </c>
       <c r="H64" t="s">
@@ -18224,9 +17477,6 @@
       <c r="F65" t="s">
         <v>258</v>
       </c>
-      <c r="G65" t="s">
-        <v>258</v>
-      </c>
       <c r="H65" t="s">
         <v>258</v>
       </c>
@@ -18283,16 +17533,10 @@
       <c r="C66" t="s">
         <v>258</v>
       </c>
-      <c r="D66" t="s">
-        <v>258</v>
-      </c>
       <c r="E66" t="s">
         <v>258</v>
       </c>
       <c r="F66" t="s">
-        <v>258</v>
-      </c>
-      <c r="G66" t="s">
         <v>258</v>
       </c>
       <c r="H66" t="s">
@@ -18354,9 +17598,6 @@
       <c r="C67" t="s">
         <v>258</v>
       </c>
-      <c r="D67" t="s">
-        <v>258</v>
-      </c>
       <c r="P67" t="s">
         <v>258</v>
       </c>
@@ -18386,16 +17627,10 @@
       <c r="C68" t="s">
         <v>258</v>
       </c>
-      <c r="D68" t="s">
-        <v>258</v>
-      </c>
       <c r="E68" t="s">
         <v>258</v>
       </c>
       <c r="F68" t="s">
-        <v>258</v>
-      </c>
-      <c r="G68" t="s">
         <v>258</v>
       </c>
       <c r="H68" t="s">
@@ -18487,9 +17722,6 @@
       <c r="Q69" t="s">
         <v>258</v>
       </c>
-      <c r="R69" t="s">
-        <v>258</v>
-      </c>
       <c r="S69" t="s">
         <v>258</v>
       </c>
@@ -18575,9 +17807,6 @@
       <c r="A71" t="s">
         <v>82</v>
       </c>
-      <c r="C71" t="s">
-        <v>258</v>
-      </c>
       <c r="D71" t="s">
         <v>258</v>
       </c>
@@ -18594,9 +17823,6 @@
         <v>258</v>
       </c>
       <c r="Q71" t="s">
-        <v>258</v>
-      </c>
-      <c r="R71" t="s">
         <v>258</v>
       </c>
       <c r="S71" t="s">
@@ -18622,9 +17848,6 @@
       <c r="C72" t="s">
         <v>258</v>
       </c>
-      <c r="D72" t="s">
-        <v>258</v>
-      </c>
       <c r="E72" t="s">
         <v>258</v>
       </c>
@@ -18690,9 +17913,6 @@
       <c r="C73" t="s">
         <v>258</v>
       </c>
-      <c r="D73" t="s">
-        <v>258</v>
-      </c>
       <c r="E73" t="s">
         <v>258</v>
       </c>
@@ -18764,9 +17984,6 @@
       <c r="F74" t="s">
         <v>258</v>
       </c>
-      <c r="G74" t="s">
-        <v>258</v>
-      </c>
       <c r="H74" t="s">
         <v>258</v>
       </c>
@@ -18832,16 +18049,10 @@
       <c r="C75" t="s">
         <v>258</v>
       </c>
-      <c r="D75" t="s">
-        <v>258</v>
-      </c>
       <c r="E75" t="s">
         <v>258</v>
       </c>
       <c r="F75" t="s">
-        <v>258</v>
-      </c>
-      <c r="G75" t="s">
         <v>258</v>
       </c>
       <c r="H75" t="s">
@@ -18903,9 +18114,6 @@
       <c r="C76" t="s">
         <v>258</v>
       </c>
-      <c r="D76" t="s">
-        <v>258</v>
-      </c>
       <c r="E76" t="s">
         <v>258</v>
       </c>
@@ -18997,21 +18205,12 @@
       <c r="B78" t="s">
         <v>258</v>
       </c>
-      <c r="C78" t="s">
-        <v>258</v>
-      </c>
-      <c r="D78" t="s">
-        <v>258</v>
-      </c>
       <c r="E78" t="s">
         <v>258</v>
       </c>
       <c r="F78" t="s">
         <v>258</v>
       </c>
-      <c r="G78" t="s">
-        <v>258</v>
-      </c>
       <c r="H78" t="s">
         <v>258</v>
       </c>
@@ -19040,9 +18239,6 @@
         <v>258</v>
       </c>
       <c r="Q78" t="s">
-        <v>258</v>
-      </c>
-      <c r="R78" t="s">
         <v>258</v>
       </c>
       <c r="S78" t="s">
@@ -19083,9 +18279,6 @@
       <c r="F79" t="s">
         <v>258</v>
       </c>
-      <c r="G79" t="s">
-        <v>258</v>
-      </c>
       <c r="H79" t="s">
         <v>258</v>
       </c>
@@ -19151,9 +18344,6 @@
       <c r="F80" t="s">
         <v>258</v>
       </c>
-      <c r="G80" t="s">
-        <v>258</v>
-      </c>
       <c r="H80" t="s">
         <v>258</v>
       </c>
@@ -19213,16 +18403,10 @@
       <c r="C81" t="s">
         <v>258</v>
       </c>
-      <c r="D81" t="s">
-        <v>258</v>
-      </c>
       <c r="E81" t="s">
         <v>258</v>
       </c>
       <c r="F81" t="s">
-        <v>258</v>
-      </c>
-      <c r="G81" t="s">
         <v>258</v>
       </c>
       <c r="H81" t="s">
@@ -19284,19 +18468,10 @@
       <c r="B82" t="s">
         <v>258</v>
       </c>
-      <c r="C82" t="s">
-        <v>258</v>
-      </c>
-      <c r="D82" t="s">
-        <v>258</v>
-      </c>
       <c r="E82" t="s">
         <v>258</v>
       </c>
       <c r="F82" t="s">
-        <v>258</v>
-      </c>
-      <c r="G82" t="s">
         <v>258</v>
       </c>
       <c r="H82" t="s">
@@ -19370,9 +18545,6 @@
       <c r="F83" t="s">
         <v>258</v>
       </c>
-      <c r="G83" t="s">
-        <v>258</v>
-      </c>
       <c r="H83" t="s">
         <v>258</v>
       </c>
@@ -19401,9 +18573,6 @@
         <v>258</v>
       </c>
       <c r="Q83" t="s">
-        <v>258</v>
-      </c>
-      <c r="R83" t="s">
         <v>258</v>
       </c>
       <c r="S83" t="s">
@@ -19441,9 +18610,6 @@
       <c r="C84" t="s">
         <v>258</v>
       </c>
-      <c r="D84" t="s">
-        <v>258</v>
-      </c>
       <c r="E84" t="s">
         <v>258</v>
       </c>
@@ -19515,9 +18681,6 @@
       <c r="F85" t="s">
         <v>258</v>
       </c>
-      <c r="G85" t="s">
-        <v>258</v>
-      </c>
       <c r="H85" t="s">
         <v>258</v>
       </c>
@@ -19586,9 +18749,6 @@
       <c r="F86" t="s">
         <v>258</v>
       </c>
-      <c r="G86" t="s">
-        <v>258</v>
-      </c>
       <c r="H86" t="s">
         <v>258</v>
       </c>
@@ -19648,16 +18808,10 @@
       <c r="C87" t="s">
         <v>258</v>
       </c>
-      <c r="D87" t="s">
-        <v>258</v>
-      </c>
       <c r="E87" t="s">
         <v>258</v>
       </c>
       <c r="F87" t="s">
-        <v>258</v>
-      </c>
-      <c r="G87" t="s">
         <v>258</v>
       </c>
       <c r="H87" t="s">
@@ -19725,9 +18879,6 @@
       <c r="F88" t="s">
         <v>258</v>
       </c>
-      <c r="G88" t="s">
-        <v>258</v>
-      </c>
       <c r="H88" t="s">
         <v>258</v>
       </c>
@@ -19784,9 +18935,6 @@
       <c r="F89" t="s">
         <v>258</v>
       </c>
-      <c r="G89" t="s">
-        <v>258</v>
-      </c>
       <c r="H89" t="s">
         <v>258</v>
       </c>
@@ -19846,16 +18994,10 @@
       <c r="C90" t="s">
         <v>258</v>
       </c>
-      <c r="D90" t="s">
-        <v>258</v>
-      </c>
       <c r="E90" t="s">
         <v>258</v>
       </c>
       <c r="F90" t="s">
-        <v>258</v>
-      </c>
-      <c r="G90" t="s">
         <v>258</v>
       </c>
       <c r="H90" t="s">
@@ -19994,9 +19136,6 @@
       <c r="F92" t="s">
         <v>258</v>
       </c>
-      <c r="G92" t="s">
-        <v>258</v>
-      </c>
       <c r="H92" t="s">
         <v>258</v>
       </c>
@@ -20062,9 +19201,6 @@
       <c r="F93" t="s">
         <v>258</v>
       </c>
-      <c r="G93" t="s">
-        <v>258</v>
-      </c>
       <c r="H93" t="s">
         <v>258</v>
       </c>
@@ -20192,16 +19328,10 @@
       <c r="C95" t="s">
         <v>258</v>
       </c>
-      <c r="D95" t="s">
-        <v>258</v>
-      </c>
       <c r="E95" t="s">
         <v>258</v>
       </c>
       <c r="F95" t="s">
-        <v>258</v>
-      </c>
-      <c r="G95" t="s">
         <v>258</v>
       </c>
       <c r="H95" t="s">
@@ -20269,9 +19399,6 @@
       <c r="F96" t="s">
         <v>258</v>
       </c>
-      <c r="G96" t="s">
-        <v>258</v>
-      </c>
       <c r="H96" t="s">
         <v>258</v>
       </c>
@@ -20325,16 +19452,10 @@
       <c r="A97" t="s">
         <v>108</v>
       </c>
-      <c r="C97" t="s">
-        <v>258</v>
-      </c>
       <c r="D97" t="s">
         <v>258</v>
       </c>
       <c r="E97" t="s">
-        <v>258</v>
-      </c>
-      <c r="G97" t="s">
         <v>258</v>
       </c>
       <c r="H97" t="s">
@@ -20396,9 +19517,6 @@
       <c r="E98" t="s">
         <v>258</v>
       </c>
-      <c r="G98" t="s">
-        <v>258</v>
-      </c>
       <c r="H98" t="s">
         <v>258</v>
       </c>
@@ -20449,16 +19567,10 @@
       <c r="C99" t="s">
         <v>258</v>
       </c>
-      <c r="D99" t="s">
-        <v>258</v>
-      </c>
       <c r="E99" t="s">
         <v>258</v>
       </c>
       <c r="F99" t="s">
-        <v>258</v>
-      </c>
-      <c r="G99" t="s">
         <v>258</v>
       </c>
       <c r="H99" t="s">
@@ -20526,9 +19638,6 @@
       <c r="C100" t="s">
         <v>258</v>
       </c>
-      <c r="D100" t="s">
-        <v>258</v>
-      </c>
       <c r="E100" t="s">
         <v>258</v>
       </c>
@@ -20597,9 +19706,6 @@
       <c r="F101" t="s">
         <v>258</v>
       </c>
-      <c r="G101" t="s">
-        <v>258</v>
-      </c>
       <c r="H101" t="s">
         <v>258</v>
       </c>
@@ -20628,9 +19734,6 @@
         <v>258</v>
       </c>
       <c r="Q101" t="s">
-        <v>258</v>
-      </c>
-      <c r="R101" t="s">
         <v>258</v>
       </c>
       <c r="S101" t="s">
@@ -20677,9 +19780,6 @@
       <c r="F102" t="s">
         <v>258</v>
       </c>
-      <c r="G102" t="s">
-        <v>258</v>
-      </c>
       <c r="H102" t="s">
         <v>258</v>
       </c>
@@ -20742,16 +19842,10 @@
       <c r="C103" t="s">
         <v>258</v>
       </c>
-      <c r="D103" t="s">
-        <v>258</v>
-      </c>
       <c r="E103" t="s">
         <v>258</v>
       </c>
       <c r="F103" t="s">
-        <v>258</v>
-      </c>
-      <c r="G103" t="s">
         <v>258</v>
       </c>
       <c r="H103" t="s">
@@ -20819,16 +19913,10 @@
       <c r="C104" t="s">
         <v>258</v>
       </c>
-      <c r="D104" t="s">
-        <v>258</v>
-      </c>
       <c r="E104" t="s">
         <v>258</v>
       </c>
       <c r="F104" t="s">
-        <v>258</v>
-      </c>
-      <c r="G104" t="s">
         <v>258</v>
       </c>
       <c r="H104" t="s">
@@ -20887,16 +19975,10 @@
       <c r="A105" t="s">
         <v>116</v>
       </c>
-      <c r="C105" t="s">
-        <v>258</v>
-      </c>
       <c r="D105" t="s">
         <v>258</v>
       </c>
       <c r="E105" t="s">
-        <v>258</v>
-      </c>
-      <c r="G105" t="s">
         <v>258</v>
       </c>
       <c r="H105" t="s">
@@ -20952,9 +20034,6 @@
       <c r="F106" t="s">
         <v>258</v>
       </c>
-      <c r="G106" t="s">
-        <v>258</v>
-      </c>
       <c r="H106" t="s">
         <v>258</v>
       </c>
@@ -21073,16 +20152,10 @@
       <c r="C108" t="s">
         <v>258</v>
       </c>
-      <c r="D108" t="s">
-        <v>258</v>
-      </c>
       <c r="E108" t="s">
         <v>258</v>
       </c>
       <c r="F108" t="s">
-        <v>258</v>
-      </c>
-      <c r="G108" t="s">
         <v>258</v>
       </c>
       <c r="H108" t="s">
@@ -21147,19 +20220,10 @@
       <c r="B109" t="s">
         <v>258</v>
       </c>
-      <c r="C109" t="s">
-        <v>258</v>
-      </c>
-      <c r="D109" t="s">
-        <v>258</v>
-      </c>
       <c r="E109" t="s">
         <v>258</v>
       </c>
       <c r="F109" t="s">
-        <v>258</v>
-      </c>
-      <c r="G109" t="s">
         <v>258</v>
       </c>
       <c r="H109" t="s">
@@ -21227,16 +20291,10 @@
       <c r="C110" t="s">
         <v>258</v>
       </c>
-      <c r="D110" t="s">
-        <v>258</v>
-      </c>
       <c r="E110" t="s">
         <v>258</v>
       </c>
       <c r="F110" t="s">
-        <v>258</v>
-      </c>
-      <c r="G110" t="s">
         <v>258</v>
       </c>
       <c r="H110" t="s">
@@ -21372,16 +20430,10 @@
       <c r="C112" t="s">
         <v>258</v>
       </c>
-      <c r="D112" t="s">
-        <v>258</v>
-      </c>
       <c r="E112" t="s">
         <v>258</v>
       </c>
       <c r="F112" t="s">
-        <v>258</v>
-      </c>
-      <c r="G112" t="s">
         <v>258</v>
       </c>
       <c r="H112" t="s">
@@ -21452,16 +20504,10 @@
       <c r="C113" t="s">
         <v>258</v>
       </c>
-      <c r="D113" t="s">
-        <v>258</v>
-      </c>
       <c r="E113" t="s">
         <v>258</v>
       </c>
       <c r="F113" t="s">
-        <v>258</v>
-      </c>
-      <c r="G113" t="s">
         <v>258</v>
       </c>
       <c r="H113" t="s">
@@ -21529,15 +20575,9 @@
       <c r="C114" t="s">
         <v>258</v>
       </c>
-      <c r="D114" t="s">
-        <v>258</v>
-      </c>
       <c r="E114" t="s">
         <v>258</v>
       </c>
-      <c r="G114" t="s">
-        <v>258</v>
-      </c>
       <c r="H114" t="s">
         <v>258</v>
       </c>
@@ -21563,9 +20603,6 @@
         <v>258</v>
       </c>
       <c r="Q114" t="s">
-        <v>258</v>
-      </c>
-      <c r="R114" t="s">
         <v>258</v>
       </c>
       <c r="S114" t="s">
@@ -21600,18 +20637,12 @@
       <c r="C115" t="s">
         <v>258</v>
       </c>
-      <c r="D115" t="s">
-        <v>258</v>
-      </c>
       <c r="E115" t="s">
         <v>258</v>
       </c>
       <c r="F115" t="s">
         <v>258</v>
       </c>
-      <c r="G115" t="s">
-        <v>258</v>
-      </c>
       <c r="H115" t="s">
         <v>258</v>
       </c>
@@ -21640,9 +20671,6 @@
         <v>258</v>
       </c>
       <c r="Q115" t="s">
-        <v>258</v>
-      </c>
-      <c r="R115" t="s">
         <v>258</v>
       </c>
       <c r="S115" t="s">
@@ -21690,178 +20718,178 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>6</v>
       </c>
       <c r="C2">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="B3">
         <v>6</v>
       </c>
       <c r="C3">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="B4">
         <v>6</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>104</v>
       </c>
       <c r="B5">
         <v>6</v>
       </c>
       <c r="C5">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="B6">
         <v>6</v>
       </c>
       <c r="C6">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>6</v>
       </c>
       <c r="C8">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B9">
         <v>6</v>
       </c>
       <c r="C9">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B10">
         <v>6</v>
       </c>
       <c r="C10">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="B11">
         <v>6</v>
       </c>
       <c r="C11">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B12">
         <v>6</v>
       </c>
       <c r="C12">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B13">
         <v>6</v>
       </c>
       <c r="C13">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B14">
         <v>6</v>
       </c>
       <c r="C14">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B15">
         <v>6</v>
       </c>
       <c r="C15">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="B16">
         <v>6</v>
       </c>
       <c r="C16">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -21872,491 +20900,491 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B19">
         <v>6</v>
       </c>
       <c r="C19">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B20">
         <v>6</v>
       </c>
       <c r="C20">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B22">
         <v>6</v>
       </c>
       <c r="C22">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>124</v>
       </c>
       <c r="B23">
         <v>6</v>
       </c>
       <c r="C23">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="B24">
         <v>6</v>
       </c>
       <c r="C24">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="B25">
         <v>6</v>
       </c>
       <c r="C25">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="B26">
         <v>6</v>
       </c>
       <c r="C26">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>46</v>
       </c>
       <c r="B27">
         <v>6</v>
       </c>
       <c r="C27">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="B28">
         <v>6</v>
       </c>
       <c r="C28">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="B29">
         <v>6</v>
       </c>
       <c r="C29">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B30">
         <v>6</v>
       </c>
       <c r="C30">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="B31">
         <v>6</v>
       </c>
       <c r="C31">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>9</v>
+        <v>101</v>
       </c>
       <c r="B32">
         <v>6</v>
       </c>
       <c r="C32">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="B33">
         <v>6</v>
       </c>
       <c r="C33">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="B34">
         <v>6</v>
       </c>
       <c r="C34">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>126</v>
       </c>
       <c r="B35">
         <v>6</v>
       </c>
       <c r="C35">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B36">
         <v>6</v>
       </c>
       <c r="C36">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B37">
         <v>6</v>
       </c>
       <c r="C37">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="B38">
         <v>6</v>
       </c>
       <c r="C38">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="B39">
         <v>6</v>
       </c>
       <c r="C39">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="B40">
         <v>6</v>
       </c>
       <c r="C40">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="B41">
         <v>6</v>
       </c>
       <c r="C41">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B42">
         <v>6</v>
       </c>
       <c r="C42">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="B43">
         <v>6</v>
       </c>
       <c r="C43">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="B44">
         <v>6</v>
       </c>
       <c r="C44">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="B45">
         <v>6</v>
       </c>
       <c r="C45">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="B46">
         <v>6</v>
       </c>
       <c r="C46">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>115</v>
+        <v>74</v>
       </c>
       <c r="B47">
         <v>6</v>
       </c>
       <c r="C47">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="B48">
         <v>6</v>
       </c>
       <c r="C48">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="B49">
         <v>6</v>
       </c>
       <c r="C49">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="B50">
         <v>6</v>
       </c>
       <c r="C50">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="B51">
         <v>6</v>
       </c>
       <c r="C51">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>111</v>
       </c>
       <c r="B52">
         <v>6</v>
       </c>
       <c r="C52">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>115</v>
       </c>
       <c r="B53">
         <v>6</v>
       </c>
       <c r="C53">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="B54">
         <v>6</v>
       </c>
       <c r="C54">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="B55">
         <v>6</v>
       </c>
       <c r="C55">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B56">
         <v>6</v>
       </c>
       <c r="C56">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="B57">
         <v>6</v>
       </c>
       <c r="C57">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B58">
         <v>6</v>
       </c>
       <c r="C58">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>33</v>
+        <v>125</v>
       </c>
       <c r="B59">
         <v>6</v>
       </c>
       <c r="C59">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B60">
         <v>6</v>
       </c>
       <c r="C60">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="B61">
         <v>6</v>
       </c>
       <c r="C61">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B62">
         <v>6</v>
       </c>
       <c r="C62">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -22367,7 +21395,7 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -22378,7 +21406,7 @@
         <v>6</v>
       </c>
       <c r="C64">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -22389,7 +21417,7 @@
         <v>6</v>
       </c>
       <c r="C65">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -22400,7 +21428,7 @@
         <v>6</v>
       </c>
       <c r="C66">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -22411,7 +21439,7 @@
         <v>6</v>
       </c>
       <c r="C67">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -22422,7 +21450,7 @@
         <v>6</v>
       </c>
       <c r="C68">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -22433,7 +21461,7 @@
         <v>6</v>
       </c>
       <c r="C69">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -22444,7 +21472,7 @@
         <v>6</v>
       </c>
       <c r="C70">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -22455,56 +21483,56 @@
         <v>6</v>
       </c>
       <c r="C71">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B72">
         <v>5</v>
       </c>
       <c r="C72">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="B73">
         <v>5</v>
       </c>
       <c r="C73">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B74">
         <v>5</v>
       </c>
       <c r="C74">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B75">
         <v>5</v>
       </c>
       <c r="C75">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="B76">
         <v>5</v>
@@ -22515,7 +21543,7 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="B77">
         <v>5</v>
@@ -22526,51 +21554,51 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="B78">
         <v>5</v>
       </c>
       <c r="C78">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="B79">
         <v>5</v>
       </c>
       <c r="C79">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="B80">
         <v>5</v>
       </c>
       <c r="C80">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>122</v>
+        <v>49</v>
       </c>
       <c r="B81">
         <v>5</v>
       </c>
       <c r="C81">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="B82">
         <v>5</v>
@@ -22587,7 +21615,7 @@
         <v>5</v>
       </c>
       <c r="C83">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -22598,7 +21626,7 @@
         <v>5</v>
       </c>
       <c r="C84">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -22609,7 +21637,7 @@
         <v>5</v>
       </c>
       <c r="C85">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -22620,56 +21648,56 @@
         <v>5</v>
       </c>
       <c r="C86">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="B87">
         <v>5</v>
       </c>
       <c r="C87">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B88">
         <v>5</v>
       </c>
       <c r="C88">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B89">
         <v>5</v>
       </c>
       <c r="C89">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B90">
         <v>5</v>
       </c>
       <c r="C90">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="B91">
         <v>5</v>
@@ -22680,7 +21708,7 @@
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>68</v>
+        <v>117</v>
       </c>
       <c r="B92">
         <v>5</v>
@@ -22691,51 +21719,51 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="B93">
         <v>5</v>
       </c>
       <c r="C93">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>103</v>
+        <v>37</v>
       </c>
       <c r="B94">
         <v>5</v>
       </c>
       <c r="C94">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="B95">
         <v>5</v>
       </c>
       <c r="C95">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="B96">
         <v>5</v>
       </c>
       <c r="C96">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="B97">
         <v>5</v>
@@ -22746,7 +21774,7 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>55</v>
+        <v>107</v>
       </c>
       <c r="B98">
         <v>5</v>
@@ -22757,7 +21785,7 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="B99">
         <v>5</v>
@@ -22768,29 +21796,29 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="B100">
         <v>5</v>
       </c>
       <c r="C100">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="B101">
         <v>5</v>
       </c>
       <c r="C101">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B102">
         <v>5</v>
@@ -22807,12 +21835,12 @@
         <v>5</v>
       </c>
       <c r="C103">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="B104">
         <v>5</v>
@@ -22823,35 +21851,35 @@
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="B105">
         <v>5</v>
       </c>
       <c r="C105">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>65</v>
+        <v>109</v>
       </c>
       <c r="B106">
         <v>5</v>
       </c>
       <c r="C106">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="B107">
         <v>5</v>
       </c>
       <c r="C107">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -22873,34 +21901,34 @@
         <v>4</v>
       </c>
       <c r="C109">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B110">
         <v>4</v>
       </c>
       <c r="C110">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B111">
         <v>4</v>
       </c>
       <c r="C111">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="B112">
         <v>4</v>
@@ -22911,24 +21939,24 @@
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="B113">
         <v>4</v>
       </c>
       <c r="C113">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B114">
         <v>4</v>
       </c>
       <c r="C114">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="115" spans="1:3">

</xml_diff>